<commit_message>
feat(auth): redesign login page to match SGS mockup with full-bleed backdrop and value showcase
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F53"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1469,9 +1469,49 @@
         <v>* [COMPLETED] TSK-ATT-032 (Implement resilient silent re-authentication on system startup): Resolved a startup auto-login bug in the C# desktop agent application. During boot-time launch, slow local network interface connection speeds caused initial silent token refreshes to fail with network exceptions, prompting the login credentials dialog immediately. Introduced a transient network error flag to run silently in system tray during offline startup, and configured background timers and network change address listeners to trigger silent re-authentication once connection is restored.</v>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="2" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B52" s="2" t="str">
+        <v>TSK-DASH-001</v>
+      </c>
+      <c r="C52" s="2" t="str">
+        <v>Redesign Executive Dashboard UI &amp; Make Work Progress Dynamic</v>
+      </c>
+      <c r="D52" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E52" s="2" t="str">
+        <v>Overhauled Executive Dashboard UI to match executive design mockup. Built boardroom hero banner with forest green gradient, borderless topbar actions with vertical divider, 5 world clocks layout, 4 stat cards with wave backgrounds and high-contrast SVG action arrows, real-time dynamic work progress calculation with 10s ticker, compact checkin/checkout action button, and an expandable dropdown panel with day summary, break management, and activity log.</v>
+      </c>
+      <c r="F52" s="2" t="str">
+        <v>* [COMPLETED] TSK-DASH-001 (Redesign Executive Dashboard UI &amp; Make Work Progress Dynamic): Overhauled Executive Dashboard UI to match executive design mockup. Built boardroom hero banner with forest green gradient, borderless topbar actions with vertical divider, 5 world clocks layout, 4 stat cards with wave backgrounds and high-contrast SVG action arrows, real-time dynamic work progress calculation with 10s ticker, compact checkin/checkout action button, and an expandable dropdown panel with day summary, break management, and activity log.</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B53" s="2" t="str">
+        <v>TSK-AUTH-004</v>
+      </c>
+      <c r="C53" s="2" t="str">
+        <v>Redesign Login Page with SGS Branding, Full-Bleed Desk Backdrop &amp; Modern Layout</v>
+      </c>
+      <c r="D53" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E53" s="2" t="str">
+        <v>Redesigned login page to match SGS design mockup with login-bg.png full-bleed backdrop, value propositions showcase, cursive signature flourish, aligned logo and Contact HR header, and streamlined credentials card.</v>
+      </c>
+      <c r="F53" s="2" t="str">
+        <v>* [COMPLETED] TSK-AUTH-004 (Redesign Login Page with SGS Branding, Full-Bleed Desk Backdrop &amp; Modern Layout): Redesigned login page to match SGS design mockup with login-bg.png full-bleed backdrop, value propositions showcase, cursive signature flourish, aligned logo and Contact HR header, and streamlined credentials card.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F53"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2403,7 +2443,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W71"/>
+  <dimension ref="A1:W73"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -7471,9 +7511,151 @@
         <v>Successfully resolved the dashboard hero section layout rendering bug by completely overriding the .card background shorthand and disabling backdrop-filters on .dashboard-hero. Fixed C# desktop agent auto-start boot network drop resilience to suppress login prompts on slow startup connection.</v>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" s="2" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B72" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C72" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D72" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E72" s="2" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="F72" s="2" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="G72" s="2" t="str">
+        <v>Executive Redesign &amp; Dynamic Work Progress</v>
+      </c>
+      <c r="H72" s="2" t="str">
+        <v>TSK-DASH-001</v>
+      </c>
+      <c r="I72" s="2" t="str">
+        <v>Redesign Executive Dashboard UI &amp; Make Work Progress Dynamic</v>
+      </c>
+      <c r="J72" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K72" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L72" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M72" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N72" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O72" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P72" s="2">
+        <v>8</v>
+      </c>
+      <c r="Q72" s="2">
+        <v>3.5</v>
+      </c>
+      <c r="R72" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S72" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T72" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U72" s="2" t="str">
+        <v>2026-09-10</v>
+      </c>
+      <c r="V72" s="2" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="W72" s="2" t="str">
+        <v>Overhauled the Executive Dashboard UI to match Figma reference mockup (boardroom hero banner, borderless topbar actions with divider, 5 world clocks, 4 stat cards with wave backgrounds and high-contrast SVG arrows, dynamic work progress tracking with compact checkin/checkout, and expandable dropdown with day summary, break management, and activity log). Completed full login page visual redesign matching SGS design mockup with login-bg.png full-bleed backdrop, value propositions showcase, cursive signature flourish, aligned logo and Contact HR header, and streamlined credentials card.</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B73" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C73" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D73" s="2" t="str">
+        <v>Sprint 3</v>
+      </c>
+      <c r="E73" s="2" t="str">
+        <v>Login Page</v>
+      </c>
+      <c r="F73" s="2" t="str">
+        <v>Authentication</v>
+      </c>
+      <c r="G73" s="2" t="str">
+        <v>Login UI Redesign &amp; SGS Rebranding</v>
+      </c>
+      <c r="H73" s="2" t="str">
+        <v>TSK-AUTH-004</v>
+      </c>
+      <c r="I73" s="2" t="str">
+        <v>Redesign login page with SGS branding, full-bleed desk scene backdrop, and modern value showcase</v>
+      </c>
+      <c r="J73" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K73" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="L73" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="M73" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="N73" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O73" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P73" s="2">
+        <v>6</v>
+      </c>
+      <c r="Q73" s="2">
+        <v>3.5</v>
+      </c>
+      <c r="R73" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S73" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T73" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U73" s="2" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="V73" s="2" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="W73" s="2" t="str">
+        <v>Overhauled the Executive Dashboard UI to match Figma reference mockup (boardroom hero banner, borderless topbar actions with divider, 5 world clocks, 4 stat cards with wave backgrounds and high-contrast SVG arrows, dynamic work progress tracking with compact checkin/checkout, and expandable dropdown with day summary, break management, and activity log). Completed full login page visual redesign matching SGS design mockup with login-bg.png full-bleed backdrop, value propositions showcase, cursive signature flourish, aligned logo and Contact HR header, and streamlined credentials card.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W71"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W73"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(employees): redesign employee profile page to match executive design mockup
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F54"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1509,9 +1509,29 @@
         <v>* [COMPLETED] TSK-AUTH-004 (Redesign Login Page with SGS Branding, Full-Bleed Desk Backdrop &amp; Modern Layout): Redesigned login page to match SGS design mockup with login-bg.png full-bleed backdrop, value propositions showcase, cursive signature flourish, aligned logo and Contact HR header, and streamlined credentials card.</v>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="2" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B54" s="2" t="str">
+        <v>TSK-EMP-015</v>
+      </c>
+      <c r="C54" s="2" t="str">
+        <v>Redesign Employee Profile Page to Match Executive Design Mockup</v>
+      </c>
+      <c r="D54" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E54" s="2" t="str">
+        <v>Overhauled the Employee Profile page to match the executive design mockup. Added breadcrumb navigation, More Actions dropdown, warm golden bronze Chat button linking to Google Chat, hero card with dark navy avatar, SSG employee code chip, bold name, ACTIVE pill, subtitle, inspirational quote, 3-column stats with dynamic Years With Us, 4-column contact strip, floating pill navigation tabs with Lucide icons, and 2x2 overview details cards grid with Edit buttons and alternating zebra-striped rows.</v>
+      </c>
+      <c r="F54" s="2" t="str">
+        <v>* [COMPLETED] TSK-EMP-015 (Redesign Employee Profile Page to Match Executive Design Mockup): Overhauled the Employee Profile page to match the executive design mockup. Added breadcrumb navigation, More Actions dropdown, warm golden bronze Chat button linking to Google Chat, hero card with dark navy avatar, SSG employee code chip, bold name, ACTIVE pill, subtitle, inspirational quote, 3-column stats with dynamic Years With Us, 4-column contact strip, floating pill navigation tabs with Lucide icons, and 2x2 overview details cards grid with Edit buttons and alternating zebra-striped rows.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F53"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F54"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2443,7 +2463,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W73"/>
+  <dimension ref="A1:W74"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -7561,7 +7581,7 @@
         <v>8</v>
       </c>
       <c r="Q72" s="2">
-        <v>3.5</v>
+        <v>3.3333333333333335</v>
       </c>
       <c r="R72" s="2" t="str">
         <v>100%</v>
@@ -7579,7 +7599,7 @@
         <v>2026-09-11</v>
       </c>
       <c r="W72" s="2" t="str">
-        <v>Overhauled the Executive Dashboard UI to match Figma reference mockup (boardroom hero banner, borderless topbar actions with divider, 5 world clocks, 4 stat cards with wave backgrounds and high-contrast SVG arrows, dynamic work progress tracking with compact checkin/checkout, and expandable dropdown with day summary, break management, and activity log). Completed full login page visual redesign matching SGS design mockup with login-bg.png full-bleed backdrop, value propositions showcase, cursive signature flourish, aligned logo and Contact HR header, and streamlined credentials card.</v>
+        <v>Overhauled the Executive Dashboard UI to match Figma reference mockup and completed full login page visual redesign. Redesigned Employee Profile page to match executive design mockup with breadcrumb header, More Actions dropdown, golden bronze Chat button, hero card with dark navy avatar, SSG employee code chip, bold name, ACTIVE pill, subtitle, quote, 3-column stats with dynamic Years With Us, 4-column contact strip, floating pill navigation tabs with Lucide icons, and 2x2 overview details cards grid with Edit buttons and alternating zebra-striped rows.</v>
       </c>
     </row>
     <row r="73">
@@ -7632,7 +7652,7 @@
         <v>6</v>
       </c>
       <c r="Q73" s="2">
-        <v>3.5</v>
+        <v>3.3333333333333335</v>
       </c>
       <c r="R73" s="2" t="str">
         <v>100%</v>
@@ -7650,12 +7670,83 @@
         <v>2026-09-11</v>
       </c>
       <c r="W73" s="2" t="str">
-        <v>Overhauled the Executive Dashboard UI to match Figma reference mockup (boardroom hero banner, borderless topbar actions with divider, 5 world clocks, 4 stat cards with wave backgrounds and high-contrast SVG arrows, dynamic work progress tracking with compact checkin/checkout, and expandable dropdown with day summary, break management, and activity log). Completed full login page visual redesign matching SGS design mockup with login-bg.png full-bleed backdrop, value propositions showcase, cursive signature flourish, aligned logo and Contact HR header, and streamlined credentials card.</v>
+        <v>Overhauled the Executive Dashboard UI to match Figma reference mockup and completed full login page visual redesign. Redesigned Employee Profile page to match executive design mockup with breadcrumb header, More Actions dropdown, golden bronze Chat button, hero card with dark navy avatar, SSG employee code chip, bold name, ACTIVE pill, subtitle, quote, 3-column stats with dynamic Years With Us, 4-column contact strip, floating pill navigation tabs with Lucide icons, and 2x2 overview details cards grid with Edit buttons and alternating zebra-striped rows.</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="B74" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C74" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D74" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E74" s="2" t="str">
+        <v>Employee Profile Page</v>
+      </c>
+      <c r="F74" s="2" t="str">
+        <v>Employees</v>
+      </c>
+      <c r="G74" s="2" t="str">
+        <v>Profile UI Redesign</v>
+      </c>
+      <c r="H74" s="2" t="str">
+        <v>TSK-EMP-015</v>
+      </c>
+      <c r="I74" s="2" t="str">
+        <v>Redesign Employee Profile Page to Match Executive Design Mockup</v>
+      </c>
+      <c r="J74" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K74" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="L74" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M74" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N74" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O74" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P74" s="2">
+        <v>6</v>
+      </c>
+      <c r="Q74" s="2">
+        <v>3.3333333333333335</v>
+      </c>
+      <c r="R74" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S74" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T74" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U74" s="2" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="V74" s="2" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="W74" s="2" t="str">
+        <v>Overhauled the Executive Dashboard UI to match Figma reference mockup and completed full login page visual redesign. Redesigned Employee Profile page to match executive design mockup with breadcrumb header, More Actions dropdown, golden bronze Chat button, hero card with dark navy avatar, SSG employee code chip, bold name, ACTIVE pill, subtitle, quote, 3-column stats with dynamic Years With Us, 4-column contact strip, floating pill navigation tabs with Lucide icons, and 2x2 overview details cards grid with Edit buttons and alternating zebra-striped rows.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W73"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W74"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>